<commit_message>
Final update of codes - 18/09/2026
</commit_message>
<xml_diff>
--- a/deterministic_data.xlsx
+++ b/deterministic_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\OneDrive\Έγγραφα\python\Deterministic-optimization-problem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8ecc8d9ed5a21f5e/Έγγραφα/python/MS-Thesis-Codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ED31F5A-1865-4297-B1AE-7DD5FFD2DA8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="78" documentId="13_ncr:1_{1B0BCB34-AB88-4A3A-9C66-924534454A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7294374-9BAC-4A6B-AD96-07F10E3FB9A8}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{3BAA5D3A-7CAC-420F-A88F-653F0B126F94}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{3BAA5D3A-7CAC-420F-A88F-653F0B126F94}"/>
   </bookViews>
   <sheets>
     <sheet name="Orders" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="34">
   <si>
     <t>order_id</t>
   </si>
@@ -49,9 +49,6 @@
     <t>type</t>
   </si>
   <si>
-    <t>profit (€)</t>
-  </si>
-  <si>
     <t>duration (h)</t>
   </si>
   <si>
@@ -140,6 +137,9 @@
   </si>
   <si>
     <t>compatible_order_types</t>
+  </si>
+  <si>
+    <t>revenue (€)</t>
   </si>
   <si>
     <t>C</t>
@@ -223,6 +223,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -522,7 +526,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA70E7C4-CA59-47DC-B987-1B0598354D17}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultColWidth="20" defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -539,7 +543,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -547,16 +551,16 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C2" s="2">
-        <v>1000</v>
+        <v>8</v>
       </c>
       <c r="D2" s="2">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="E2" s="2">
-        <v>1</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -564,16 +568,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C3" s="3">
-        <v>2000</v>
+        <v>2</v>
       </c>
       <c r="D3" s="3">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="E3" s="3">
-        <v>2</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -581,16 +585,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C4" s="2">
-        <v>2500</v>
+        <v>5</v>
       </c>
       <c r="D4" s="2">
-        <v>5</v>
+        <v>300</v>
       </c>
       <c r="E4" s="2">
-        <v>1</v>
+        <v>120200</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -598,16 +602,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5" s="3">
-        <v>1500</v>
+        <v>4</v>
       </c>
       <c r="D5" s="3">
-        <v>3</v>
+        <v>64</v>
       </c>
       <c r="E5" s="3">
-        <v>2</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -615,16 +619,50 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2">
         <v>6</v>
       </c>
-      <c r="C6" s="2">
-        <v>0</v>
-      </c>
       <c r="D6" s="2">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="E6" s="2">
-        <v>1</v>
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3">
+        <v>32</v>
+      </c>
+      <c r="E7" s="3">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="2">
+        <v>8</v>
+      </c>
+      <c r="D8" s="2">
+        <v>32</v>
+      </c>
+      <c r="E8" s="2">
+        <v>50000</v>
       </c>
     </row>
   </sheetData>
@@ -639,13 +677,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -653,10 +691,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -664,10 +702,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -678,7 +716,7 @@
         <v>33</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -693,150 +731,150 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="X1" s="1" t="s">
-        <v>30</v>
-      </c>
     </row>
     <row r="2" spans="1:24" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3">
-        <v>152</v>
-      </c>
-      <c r="B2" s="3">
-        <v>156</v>
-      </c>
-      <c r="C2" s="3">
-        <v>70</v>
-      </c>
-      <c r="D2" s="3">
-        <v>156</v>
-      </c>
-      <c r="E2" s="3">
-        <v>189</v>
-      </c>
-      <c r="F2" s="3">
-        <v>195</v>
-      </c>
-      <c r="G2" s="3">
-        <v>119</v>
-      </c>
-      <c r="H2" s="3">
-        <v>129</v>
-      </c>
-      <c r="I2" s="3">
-        <v>125</v>
-      </c>
-      <c r="J2" s="3">
-        <v>156</v>
-      </c>
-      <c r="K2" s="3">
-        <v>97</v>
-      </c>
-      <c r="L2" s="3">
-        <v>242</v>
-      </c>
-      <c r="M2" s="3">
-        <v>92</v>
-      </c>
-      <c r="N2" s="3">
-        <v>197</v>
-      </c>
-      <c r="O2" s="3">
-        <v>159</v>
-      </c>
-      <c r="P2" s="3">
-        <v>142</v>
-      </c>
-      <c r="Q2" s="3">
-        <v>113</v>
-      </c>
-      <c r="R2" s="3">
-        <v>91</v>
-      </c>
-      <c r="S2" s="3">
-        <v>209</v>
-      </c>
-      <c r="T2" s="3">
-        <v>211</v>
-      </c>
-      <c r="U2" s="3">
-        <v>50</v>
-      </c>
-      <c r="V2" s="3">
-        <v>247</v>
-      </c>
-      <c r="W2" s="3">
-        <v>88</v>
-      </c>
-      <c r="X2" s="3">
-        <v>209</v>
+      <c r="A2">
+        <v>92.47</v>
+      </c>
+      <c r="B2">
+        <v>88.48</v>
+      </c>
+      <c r="C2">
+        <v>84.92</v>
+      </c>
+      <c r="D2">
+        <v>80.23</v>
+      </c>
+      <c r="E2">
+        <v>77.61</v>
+      </c>
+      <c r="F2">
+        <v>79.489999999999995</v>
+      </c>
+      <c r="G2">
+        <v>86.58</v>
+      </c>
+      <c r="H2">
+        <v>97.01</v>
+      </c>
+      <c r="I2">
+        <v>103.52</v>
+      </c>
+      <c r="J2">
+        <v>98.86</v>
+      </c>
+      <c r="K2">
+        <v>89.75</v>
+      </c>
+      <c r="L2">
+        <v>83.22</v>
+      </c>
+      <c r="M2">
+        <v>80.06</v>
+      </c>
+      <c r="N2">
+        <v>79.36</v>
+      </c>
+      <c r="O2">
+        <v>77.19</v>
+      </c>
+      <c r="P2">
+        <v>81.38</v>
+      </c>
+      <c r="Q2">
+        <v>90.19</v>
+      </c>
+      <c r="R2">
+        <v>101.53</v>
+      </c>
+      <c r="S2">
+        <v>112.2</v>
+      </c>
+      <c r="T2">
+        <v>121.08</v>
+      </c>
+      <c r="U2">
+        <v>128.68</v>
+      </c>
+      <c r="V2">
+        <v>122.59</v>
+      </c>
+      <c r="W2">
+        <v>107.84</v>
+      </c>
+      <c r="X2">
+        <v>100.24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>